<commit_message>
Extend the project title to be longer than 20 characters in metadata files
</commit_message>
<xml_diff>
--- a/tests/resources/metadata_files/EVA_Submission_v1.1.4_cpombe.xlsx
+++ b/tests/resources/metadata_files/EVA_Submission_v1.1.4_cpombe.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10824"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10419"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tcezard/PycharmProjects/eva-integration-tests/tests/resources/metadata_spreadsheets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tcezard/PycharmProjects/eva-integration-tests/tests/resources/metadata_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95F9D495-CD53-4E41-BBAA-B9D9BD0879D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{761B87E1-E7DE-4242-95E1-25315242954C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16020" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="60160" yWindow="680" windowWidth="28800" windowHeight="16020" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLEASE READ FIRST" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="741" uniqueCount="578">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="741" uniqueCount="579">
   <si>
     <t>PLEASE READ FIRST</t>
   </si>
@@ -1913,6 +1913,9 @@
   </si>
   <si>
     <t>VCF</t>
+  </si>
+  <si>
+    <t>test_project_title_a_bit_longer</t>
   </si>
 </sst>
 </file>
@@ -2446,18 +2449,7 @@
     <xf numFmtId="164" fontId="21" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="21" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2467,8 +2459,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2482,7 +2486,6 @@
     <xf numFmtId="0" fontId="17" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2843,8 +2846,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="62"/>
-      <c r="B1" s="62"/>
+      <c r="A1" s="67"/>
+      <c r="B1" s="67"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
@@ -2853,10 +2856,10 @@
       <c r="H1" s="2"/>
     </row>
     <row r="2" spans="1:8" s="3" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="69" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="63"/>
+      <c r="B2" s="69"/>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -2865,10 +2868,10 @@
       <c r="H2" s="4"/>
     </row>
     <row r="3" spans="1:8" s="3" customFormat="1" ht="19" x14ac:dyDescent="0.25">
-      <c r="A3" s="64" t="s">
+      <c r="A3" s="70" t="s">
         <v>523</v>
       </c>
-      <c r="B3" s="64"/>
+      <c r="B3" s="70"/>
       <c r="C3" s="5"/>
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
@@ -2877,10 +2880,10 @@
       <c r="H3" s="5"/>
     </row>
     <row r="4" spans="1:8" s="3" customFormat="1" ht="19" x14ac:dyDescent="0.25">
-      <c r="A4" s="65" t="s">
+      <c r="A4" s="66" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="65"/>
+      <c r="B4" s="66"/>
       <c r="C4" s="6"/>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
@@ -2889,8 +2892,8 @@
       <c r="H4" s="6"/>
     </row>
     <row r="5" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="62"/>
-      <c r="B5" s="62"/>
+      <c r="A5" s="67"/>
+      <c r="B5" s="67"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
@@ -2911,10 +2914,10 @@
       <c r="H6" s="6"/>
     </row>
     <row r="7" spans="1:8" s="3" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="67" t="s">
+      <c r="A7" s="64" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="67"/>
+      <c r="B7" s="64"/>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
       <c r="E7" s="7"/>
@@ -2923,8 +2926,8 @@
       <c r="H7" s="7"/>
     </row>
     <row r="8" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="68"/>
-      <c r="B8" s="68"/>
+      <c r="A8" s="65"/>
+      <c r="B8" s="65"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
@@ -2933,10 +2936,10 @@
       <c r="H8" s="2"/>
     </row>
     <row r="9" spans="1:8" s="3" customFormat="1" ht="19" x14ac:dyDescent="0.25">
-      <c r="A9" s="65" t="s">
+      <c r="A9" s="66" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="65"/>
+      <c r="B9" s="66"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
@@ -2945,8 +2948,8 @@
       <c r="H9" s="2"/>
     </row>
     <row r="10" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="62"/>
-      <c r="B10" s="62"/>
+      <c r="A10" s="67"/>
+      <c r="B10" s="67"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
@@ -2955,10 +2958,10 @@
       <c r="H10" s="2"/>
     </row>
     <row r="11" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="69" t="s">
+      <c r="A11" s="68" t="s">
         <v>518</v>
       </c>
-      <c r="B11" s="69"/>
+      <c r="B11" s="68"/>
     </row>
     <row r="12" spans="1:8" ht="20" x14ac:dyDescent="0.2">
       <c r="A12" s="25" t="s">
@@ -3014,28 +3017,28 @@
       <c r="B18"/>
     </row>
     <row r="19" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="66" t="s">
+      <c r="A19" s="63" t="s">
         <v>12</v>
       </c>
-      <c r="B19" s="66"/>
+      <c r="B19" s="63"/>
     </row>
     <row r="20" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="66" t="s">
+      <c r="A20" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="66"/>
+      <c r="B20" s="63"/>
     </row>
     <row r="21" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="66" t="s">
+      <c r="A21" s="63" t="s">
         <v>14</v>
       </c>
-      <c r="B21" s="66"/>
+      <c r="B21" s="63"/>
     </row>
     <row r="22" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="66" t="s">
+      <c r="A22" s="63" t="s">
         <v>15</v>
       </c>
-      <c r="B22" s="66"/>
+      <c r="B22" s="63"/>
     </row>
     <row r="23" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A23" s="10"/>
@@ -3044,6 +3047,11 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="qXS9mSszo6ZK4PVLf2a4mgrLN9LTYf+uHOdaWY7gal7eLQi1TYc4PKeNVhIGj1PsRxEc/Fk3JaqC7G3YqwmFZQ==" saltValue="v8qTKlsQPInt8A+7GIueog==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="14">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:B5"/>
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A21:B21"/>
@@ -3053,11 +3061,6 @@
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A5:B5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -5124,7 +5127,7 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>565</v>
+        <v>578</v>
       </c>
       <c r="B2" t="s">
         <v>568</v>
@@ -6212,12 +6215,12 @@
   <sheetData>
     <row r="1" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A1" s="51"/>
-      <c r="B1" s="71" t="s">
+      <c r="B1" s="72" t="s">
         <v>153</v>
       </c>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="72"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="73"/>
       <c r="F1" s="38" t="s">
         <v>154</v>
       </c>
@@ -6264,64 +6267,64 @@
     </row>
     <row r="2" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A2" s="52"/>
-      <c r="B2" s="71"/>
-      <c r="C2" s="71"/>
-      <c r="D2" s="71"/>
-      <c r="E2" s="72"/>
-      <c r="F2" s="70" t="s">
+      <c r="B2" s="72"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="73"/>
+      <c r="F2" s="71" t="s">
         <v>64</v>
       </c>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
-      <c r="K2" s="70"/>
-      <c r="L2" s="73" t="s">
+      <c r="G2" s="71"/>
+      <c r="H2" s="71"/>
+      <c r="I2" s="71"/>
+      <c r="J2" s="71"/>
+      <c r="K2" s="71"/>
+      <c r="L2" s="74" t="s">
         <v>76</v>
       </c>
-      <c r="M2" s="73"/>
-      <c r="N2" s="73"/>
-      <c r="O2" s="73" t="s">
+      <c r="M2" s="74"/>
+      <c r="N2" s="74"/>
+      <c r="O2" s="74" t="s">
         <v>83</v>
       </c>
-      <c r="P2" s="73"/>
-      <c r="Q2" s="73"/>
-      <c r="R2" s="70" t="s">
+      <c r="P2" s="74"/>
+      <c r="Q2" s="74"/>
+      <c r="R2" s="71" t="s">
         <v>88</v>
       </c>
-      <c r="S2" s="70"/>
-      <c r="T2" s="70"/>
-      <c r="U2" s="70"/>
-      <c r="V2" s="70"/>
-      <c r="W2" s="70" t="s">
+      <c r="S2" s="71"/>
+      <c r="T2" s="71"/>
+      <c r="U2" s="71"/>
+      <c r="V2" s="71"/>
+      <c r="W2" s="71" t="s">
         <v>99</v>
       </c>
-      <c r="X2" s="70"/>
-      <c r="Y2" s="70"/>
-      <c r="Z2" s="70" t="s">
+      <c r="X2" s="71"/>
+      <c r="Y2" s="71"/>
+      <c r="Z2" s="71" t="s">
         <v>106</v>
       </c>
-      <c r="AA2" s="70"/>
-      <c r="AB2" s="70"/>
-      <c r="AC2" s="70"/>
-      <c r="AD2" s="70"/>
-      <c r="AE2" s="70"/>
-      <c r="AF2" s="70"/>
-      <c r="AG2" s="70"/>
-      <c r="AH2" s="70"/>
-      <c r="AI2" s="70"/>
-      <c r="AJ2" s="70" t="s">
+      <c r="AA2" s="71"/>
+      <c r="AB2" s="71"/>
+      <c r="AC2" s="71"/>
+      <c r="AD2" s="71"/>
+      <c r="AE2" s="71"/>
+      <c r="AF2" s="71"/>
+      <c r="AG2" s="71"/>
+      <c r="AH2" s="71"/>
+      <c r="AI2" s="71"/>
+      <c r="AJ2" s="71" t="s">
         <v>127</v>
       </c>
-      <c r="AK2" s="70"/>
-      <c r="AL2" s="70"/>
-      <c r="AM2" s="70"/>
-      <c r="AN2" s="70"/>
-      <c r="AO2" s="70"/>
-      <c r="AP2" s="70"/>
-      <c r="AQ2" s="70"/>
-      <c r="AR2" s="70"/>
-      <c r="AS2" s="70"/>
+      <c r="AK2" s="71"/>
+      <c r="AL2" s="71"/>
+      <c r="AM2" s="71"/>
+      <c r="AN2" s="71"/>
+      <c r="AO2" s="71"/>
+      <c r="AP2" s="71"/>
+      <c r="AQ2" s="71"/>
+      <c r="AR2" s="71"/>
+      <c r="AS2" s="71"/>
     </row>
     <row r="3" spans="1:46" ht="26" x14ac:dyDescent="0.3">
       <c r="A3" s="39" t="s">
@@ -6479,7 +6482,7 @@
       <c r="L4">
         <v>4896</v>
       </c>
-      <c r="M4" s="74" t="s">
+      <c r="M4" s="62" t="s">
         <v>575</v>
       </c>
       <c r="Y4" s="32"/>

</xml_diff>